<commit_message>
Added setting to limit the number of afternoon shift for people in training
</commit_message>
<xml_diff>
--- a/desiderata_NOV.xlsx
+++ b/desiderata_NOV.xlsx
@@ -1,6 +1,6 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" mc:Ignorable="x15 xr xr6 xr10">
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
   <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="20417"/>
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\seria\Desktop\Repositories\shifter\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{F472AD11-EA83-48FC-89B0-AA44FEAAC445}" xr6:coauthVersionLast="36" xr6:coauthVersionMax="36" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{7D5B14B1-6C92-44BD-AED2-3916AF3EDCD8}" xr6:coauthVersionLast="36" xr6:coauthVersionMax="36" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="0" windowWidth="26835" windowHeight="12060"/>
+    <workbookView xWindow="0" yWindow="0" windowWidth="26835" windowHeight="12060" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="desiderata_NOV" sheetId="1" r:id="rId1"/>
@@ -20,7 +20,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="30" uniqueCount="26">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="28" uniqueCount="24">
   <si>
     <t>Persona</t>
   </si>
@@ -64,46 +64,40 @@
     <t>Messana</t>
   </si>
   <si>
-    <t>5/11/2025 P, 14/11/2025 M, 18/11/2025 P, 24/11/2025 P</t>
-  </si>
-  <si>
     <t>01/11/2025, 22/11/2025</t>
   </si>
   <si>
-    <t>01/11/2025-10/11/2025</t>
-  </si>
-  <si>
     <t>Scardino</t>
   </si>
   <si>
-    <t>3/11/2025 M, 7/11/2025 P, 20/11/2025 P, 25/11/2025 P</t>
-  </si>
-  <si>
     <t>15/11/2025, 22/11/2025</t>
   </si>
   <si>
     <t>Rudenko</t>
   </si>
   <si>
-    <t>6/11/2025 P, 7/11/2025 P, 11/11/2025 P, 24/11/2025 M, 27/11/2025 P</t>
-  </si>
-  <si>
-    <t>8/11/2025, 29/11/2025</t>
-  </si>
-  <si>
     <t>Odales</t>
   </si>
   <si>
-    <t>5/11/2025 P, 13/11/2025 P, 18/11/2025 P, 24/11/2025 M, 26/11/2025 P</t>
-  </si>
-  <si>
     <t>1/11/2025, 15/11/2025</t>
+  </si>
+  <si>
+    <t>4/11/2025 P, 11/11/2025 P, 18/11/2025 P, 25/11/2025 P, 6/11/2025 MP</t>
+  </si>
+  <si>
+    <t>5/11/2025 P, 14/11/2025 P, 18/11/2025 P, 24/11/2025 P</t>
+  </si>
+  <si>
+    <t>3/11/2025 P, 7/11/2025 P, 20/11/2025 P, 25/11/2025 P</t>
+  </si>
+  <si>
+    <t>5/11/2025 P, 13/11/2025 P, 18/11/2025 P, 24/11/2025 P, 26/11/2025 P</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
-<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" mc:Ignorable="x14ac x16r2">
+<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
   <fonts count="18" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
@@ -240,7 +234,7 @@
       <scheme val="minor"/>
     </font>
   </fonts>
-  <fills count="33">
+  <fills count="34">
     <fill>
       <patternFill patternType="none"/>
     </fill>
@@ -418,6 +412,12 @@
       <patternFill patternType="solid">
         <fgColor theme="9" tint="0.39997558519241921"/>
         <bgColor indexed="65"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFFFFF00"/>
+        <bgColor indexed="64"/>
       </patternFill>
     </fill>
   </fills>
@@ -581,8 +581,9 @@
     <xf numFmtId="0" fontId="1" fillId="31" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
     <xf numFmtId="0" fontId="1" fillId="32" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="1">
+  <cellXfs count="2">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="33" borderId="0" xfId="0" applyFill="1"/>
   </cellXfs>
   <cellStyles count="42">
     <cellStyle name="20% - Accent1" xfId="19" builtinId="30" customBuiltin="1"/>
@@ -937,7 +938,7 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
   <dimension ref="A1:H6"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <sheetData>
@@ -1004,18 +1005,15 @@
         <v>1</v>
       </c>
       <c r="E3" t="s">
+        <v>21</v>
+      </c>
+      <c r="F3" t="s">
         <v>14</v>
-      </c>
-      <c r="F3" t="s">
-        <v>15</v>
-      </c>
-      <c r="G3" t="s">
-        <v>16</v>
       </c>
     </row>
     <row r="4" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
-        <v>17</v>
+        <v>15</v>
       </c>
       <c r="B4" t="s">
         <v>9</v>
@@ -1027,15 +1025,15 @@
         <v>1</v>
       </c>
       <c r="E4" t="s">
-        <v>18</v>
+        <v>22</v>
       </c>
       <c r="F4" t="s">
-        <v>19</v>
+        <v>16</v>
       </c>
     </row>
     <row r="5" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A5" t="s">
-        <v>20</v>
+        <v>17</v>
       </c>
       <c r="B5" t="s">
         <v>9</v>
@@ -1046,16 +1044,13 @@
       <c r="D5">
         <v>1</v>
       </c>
-      <c r="E5" t="s">
-        <v>21</v>
-      </c>
-      <c r="F5" t="s">
-        <v>22</v>
+      <c r="E5" s="1" t="s">
+        <v>20</v>
       </c>
     </row>
     <row r="6" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A6" t="s">
-        <v>23</v>
+        <v>18</v>
       </c>
       <c r="B6" t="s">
         <v>9</v>
@@ -1067,10 +1062,10 @@
         <v>1</v>
       </c>
       <c r="E6" t="s">
-        <v>24</v>
+        <v>23</v>
       </c>
       <c r="F6" t="s">
-        <v>25</v>
+        <v>19</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Added links to download templates in the web app
</commit_message>
<xml_diff>
--- a/desiderata_NOV.xlsx
+++ b/desiderata_NOV.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\seria\Desktop\Repositories\shifter\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{7D5B14B1-6C92-44BD-AED2-3916AF3EDCD8}" xr6:coauthVersionLast="36" xr6:coauthVersionMax="36" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{BB969E32-33BC-42B6-A046-21DF00C53677}" xr6:coauthVersionLast="36" xr6:coauthVersionMax="36" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="0" yWindow="0" windowWidth="26835" windowHeight="12060" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -20,7 +20,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="28" uniqueCount="24">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="27" uniqueCount="23">
   <si>
     <t>Persona</t>
   </si>
@@ -52,21 +52,12 @@
     <t>Y</t>
   </si>
   <si>
-    <t>3/11/2025 P, 12/11/2025 P, 14/11/2025 M, 19/11/2025 P, 21/11/2025 P</t>
-  </si>
-  <si>
-    <t>01/11/2025, 29/11/2025</t>
-  </si>
-  <si>
     <t>3/11/2025-7/11/2025,10/11/2025-14/11/2025,17/11/2025-21/11/2025,24/11/2025-28/11/2025</t>
   </si>
   <si>
     <t>Messana</t>
   </si>
   <si>
-    <t>01/11/2025, 22/11/2025</t>
-  </si>
-  <si>
     <t>Scardino</t>
   </si>
   <si>
@@ -79,19 +70,25 @@
     <t>Odales</t>
   </si>
   <si>
-    <t>1/11/2025, 15/11/2025</t>
-  </si>
-  <si>
     <t>4/11/2025 P, 11/11/2025 P, 18/11/2025 P, 25/11/2025 P, 6/11/2025 MP</t>
   </si>
   <si>
-    <t>5/11/2025 P, 14/11/2025 P, 18/11/2025 P, 24/11/2025 P</t>
-  </si>
-  <si>
-    <t>3/11/2025 P, 7/11/2025 P, 20/11/2025 P, 25/11/2025 P</t>
-  </si>
-  <si>
-    <t>5/11/2025 P, 13/11/2025 P, 18/11/2025 P, 24/11/2025 P, 26/11/2025 P</t>
+    <t>01/11/2025, 15/11/2025</t>
+  </si>
+  <si>
+    <t>5/11/2025 P, 10/11/2025 P, 19/11/2025 P, 26/11/2025 P, 17/11/2025 PN, 18/11/2025 PN</t>
+  </si>
+  <si>
+    <t>8/11/2025, 29/11/2025</t>
+  </si>
+  <si>
+    <t>7/11/2025-7/11/2025, 24/11/2025-28/11/2025</t>
+  </si>
+  <si>
+    <t>13/11/2025 P, 17/11/2025 P, 21/11/2025 P, 27/11/2025 P</t>
+  </si>
+  <si>
+    <t>4/11/2025 P, 11/11/2025 P, 20/11/2025 P, 24/11/2025 P</t>
   </si>
 </sst>
 </file>
@@ -234,7 +231,7 @@
       <scheme val="minor"/>
     </font>
   </fonts>
-  <fills count="34">
+  <fills count="35">
     <fill>
       <patternFill patternType="none"/>
     </fill>
@@ -417,6 +414,12 @@
     <fill>
       <patternFill patternType="solid">
         <fgColor rgb="FFFFFF00"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="5" tint="0.39997558519241921"/>
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
@@ -581,9 +584,11 @@
     <xf numFmtId="0" fontId="1" fillId="31" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
     <xf numFmtId="0" fontId="1" fillId="32" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="2">
+  <cellXfs count="4">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="33" borderId="0" xfId="0" applyFill="1"/>
+    <xf numFmtId="0" fontId="0" fillId="34" borderId="0" xfId="0" applyFill="1"/>
+    <xf numFmtId="14" fontId="0" fillId="34" borderId="0" xfId="0" applyNumberFormat="1" applyFill="1"/>
   </cellXfs>
   <cellStyles count="42">
     <cellStyle name="20% - Accent1" xfId="19" builtinId="30" customBuiltin="1"/>
@@ -941,6 +946,13 @@
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
   <dimension ref="A1:H6"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <cols>
+    <col min="1" max="4" width="13.42578125" customWidth="1"/>
+    <col min="5" max="5" width="79.28515625" customWidth="1"/>
+    <col min="6" max="6" width="26" customWidth="1"/>
+    <col min="7" max="7" width="22.5703125" customWidth="1"/>
+    <col min="8" max="8" width="83.5703125" customWidth="1"/>
+  </cols>
   <sheetData>
     <row r="1" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A1" t="s">
@@ -981,19 +993,20 @@
       <c r="D2">
         <v>1</v>
       </c>
-      <c r="E2" t="s">
+      <c r="E2" s="1" t="s">
+        <v>18</v>
+      </c>
+      <c r="F2" s="1" t="s">
+        <v>17</v>
+      </c>
+      <c r="G2" s="1"/>
+      <c r="H2" s="1" t="s">
         <v>10</v>
-      </c>
-      <c r="F2" t="s">
-        <v>11</v>
-      </c>
-      <c r="H2" t="s">
-        <v>12</v>
       </c>
     </row>
     <row r="3" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
-        <v>13</v>
+        <v>11</v>
       </c>
       <c r="B3" t="s">
         <v>9</v>
@@ -1004,16 +1017,18 @@
       <c r="D3">
         <v>1</v>
       </c>
-      <c r="E3" t="s">
-        <v>21</v>
-      </c>
-      <c r="F3" t="s">
-        <v>14</v>
-      </c>
+      <c r="E3" s="2" t="s">
+        <v>22</v>
+      </c>
+      <c r="F3" s="3">
+        <v>45976</v>
+      </c>
+      <c r="G3" s="2"/>
+      <c r="H3" s="2"/>
     </row>
     <row r="4" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
-        <v>15</v>
+        <v>12</v>
       </c>
       <c r="B4" t="s">
         <v>9</v>
@@ -1024,16 +1039,18 @@
       <c r="D4">
         <v>1</v>
       </c>
-      <c r="E4" t="s">
-        <v>22</v>
-      </c>
-      <c r="F4" t="s">
-        <v>16</v>
-      </c>
+      <c r="E4" s="2" t="s">
+        <v>21</v>
+      </c>
+      <c r="F4" s="2" t="s">
+        <v>13</v>
+      </c>
+      <c r="G4" s="2"/>
+      <c r="H4" s="2"/>
     </row>
     <row r="5" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A5" t="s">
-        <v>17</v>
+        <v>14</v>
       </c>
       <c r="B5" t="s">
         <v>9</v>
@@ -1045,12 +1062,15 @@
         <v>1</v>
       </c>
       <c r="E5" s="1" t="s">
-        <v>20</v>
-      </c>
+        <v>16</v>
+      </c>
+      <c r="F5" s="1"/>
+      <c r="G5" s="1"/>
+      <c r="H5" s="1"/>
     </row>
     <row r="6" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A6" t="s">
-        <v>18</v>
+        <v>15</v>
       </c>
       <c r="B6" t="s">
         <v>9</v>
@@ -1061,12 +1081,14 @@
       <c r="D6">
         <v>1</v>
       </c>
-      <c r="E6" t="s">
-        <v>23</v>
-      </c>
-      <c r="F6" t="s">
+      <c r="E6" s="1"/>
+      <c r="F6" s="1" t="s">
         <v>19</v>
       </c>
+      <c r="G6" s="1" t="s">
+        <v>20</v>
+      </c>
+      <c r="H6" s="1"/>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>

</xml_diff>

<commit_message>
Small change to desiderata test
</commit_message>
<xml_diff>
--- a/desiderata_NOV.xlsx
+++ b/desiderata_NOV.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\seria\Desktop\Repositories\shifter\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{BB969E32-33BC-42B6-A046-21DF00C53677}" xr6:coauthVersionLast="36" xr6:coauthVersionMax="36" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{3A812F6A-0336-4D73-BEA9-5095A460D030}" xr6:coauthVersionLast="36" xr6:coauthVersionMax="36" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="0" yWindow="0" windowWidth="26835" windowHeight="12060" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -76,9 +76,6 @@
     <t>01/11/2025, 15/11/2025</t>
   </si>
   <si>
-    <t>5/11/2025 P, 10/11/2025 P, 19/11/2025 P, 26/11/2025 P, 17/11/2025 PN, 18/11/2025 PN</t>
-  </si>
-  <si>
     <t>8/11/2025, 29/11/2025</t>
   </si>
   <si>
@@ -89,6 +86,9 @@
   </si>
   <si>
     <t>4/11/2025 P, 11/11/2025 P, 20/11/2025 P, 24/11/2025 P</t>
+  </si>
+  <si>
+    <t>5/11/2025 P, 14/11/2025 P, 19/11/2025 P, 26/11/2025 P, 17/11/2025 PN, 18/11/2025 PN</t>
   </si>
 </sst>
 </file>
@@ -994,7 +994,7 @@
         <v>1</v>
       </c>
       <c r="E2" s="1" t="s">
-        <v>18</v>
+        <v>22</v>
       </c>
       <c r="F2" s="1" t="s">
         <v>17</v>
@@ -1018,7 +1018,7 @@
         <v>1</v>
       </c>
       <c r="E3" s="2" t="s">
-        <v>22</v>
+        <v>21</v>
       </c>
       <c r="F3" s="3">
         <v>45976</v>
@@ -1040,7 +1040,7 @@
         <v>1</v>
       </c>
       <c r="E4" s="2" t="s">
-        <v>21</v>
+        <v>20</v>
       </c>
       <c r="F4" s="2" t="s">
         <v>13</v>
@@ -1083,10 +1083,10 @@
       </c>
       <c r="E6" s="1"/>
       <c r="F6" s="1" t="s">
+        <v>18</v>
+      </c>
+      <c r="G6" s="1" t="s">
         <v>19</v>
-      </c>
-      <c r="G6" s="1" t="s">
-        <v>20</v>
       </c>
       <c r="H6" s="1"/>
     </row>

</xml_diff>

<commit_message>
Bugfix: not covered night shift were not properly detected and reported
</commit_message>
<xml_diff>
--- a/desiderata_NOV.xlsx
+++ b/desiderata_NOV.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\seria\Desktop\Repositories\shifter\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{3A812F6A-0336-4D73-BEA9-5095A460D030}" xr6:coauthVersionLast="36" xr6:coauthVersionMax="36" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{6CB6C93F-D1A9-4332-B73B-35AAB832F65A}" xr6:coauthVersionLast="36" xr6:coauthVersionMax="36" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="0" yWindow="0" windowWidth="26835" windowHeight="12060" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -20,7 +20,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="27" uniqueCount="23">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="27" uniqueCount="24">
   <si>
     <t>Persona</t>
   </si>
@@ -89,6 +89,9 @@
   </si>
   <si>
     <t>5/11/2025 P, 14/11/2025 P, 19/11/2025 P, 26/11/2025 P, 17/11/2025 PN, 18/11/2025 PN</t>
+  </si>
+  <si>
+    <t>N</t>
   </si>
 </sst>
 </file>
@@ -985,7 +988,7 @@
         <v>8</v>
       </c>
       <c r="B2" t="s">
-        <v>9</v>
+        <v>23</v>
       </c>
       <c r="C2">
         <v>1</v>
@@ -1009,7 +1012,7 @@
         <v>11</v>
       </c>
       <c r="B3" t="s">
-        <v>9</v>
+        <v>23</v>
       </c>
       <c r="C3">
         <v>1</v>
@@ -1031,7 +1034,7 @@
         <v>12</v>
       </c>
       <c r="B4" t="s">
-        <v>9</v>
+        <v>23</v>
       </c>
       <c r="C4">
         <v>1</v>
@@ -1053,7 +1056,7 @@
         <v>14</v>
       </c>
       <c r="B5" t="s">
-        <v>9</v>
+        <v>23</v>
       </c>
       <c r="C5">
         <v>1</v>

</xml_diff>